<commit_message>
feat: move portfolio ledger to D1
</commit_message>
<xml_diff>
--- a/assets/data/Yi_Capital_HK.xlsx
+++ b/assets/data/Yi_Capital_HK.xlsx
@@ -4913,7 +4913,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J357"/>
+  <dimension ref="A1:J358"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>176312.28</v>
+        <v>176312.29</v>
       </c>
       <c r="C2" s="9" t="n">
         <v>0</v>
@@ -4996,7 +4996,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="9" t="n">
-        <v>176312.28</v>
+        <v>176312.29</v>
       </c>
       <c r="F2" s="8" t="n">
         <v>1846300</v>
@@ -5011,7 +5011,7 @@
         <v>88102</v>
       </c>
       <c r="J2" s="9" t="n">
-        <v>88210.28</v>
+        <v>88210.28999999999</v>
       </c>
     </row>
     <row r="3">
@@ -5021,7 +5021,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>170577.95</v>
+        <v>170577.93</v>
       </c>
       <c r="C3" s="9" t="n">
         <v>0</v>
@@ -5030,7 +5030,7 @@
         <v>0</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>170577.95</v>
+        <v>170577.93</v>
       </c>
       <c r="F3" s="8" t="n">
         <v>1846300</v>
@@ -5045,7 +5045,7 @@
         <v>22</v>
       </c>
       <c r="J3" s="9" t="n">
-        <v>170555.95</v>
+        <v>170555.93</v>
       </c>
     </row>
     <row r="4">
@@ -5055,7 +5055,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>171990.56</v>
+        <v>171990.57</v>
       </c>
       <c r="C4" s="9" t="n">
         <v>0</v>
@@ -5064,7 +5064,7 @@
         <v>0</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>171990.56</v>
+        <v>171990.57</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>1846300</v>
@@ -5079,7 +5079,7 @@
         <v>22</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>171968.56</v>
+        <v>171968.57</v>
       </c>
     </row>
     <row r="5">
@@ -5157,7 +5157,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>175348.44</v>
+        <v>175348.45</v>
       </c>
       <c r="C7" s="9" t="n">
         <v>0</v>
@@ -5166,7 +5166,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>175348.44</v>
+        <v>175348.45</v>
       </c>
       <c r="F7" s="8" t="n">
         <v>1846300</v>
@@ -5181,7 +5181,7 @@
         <v>22</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>175326.44</v>
+        <v>175326.45</v>
       </c>
     </row>
     <row r="8">
@@ -5225,7 +5225,7 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>247354.82</v>
+        <v>247354.83</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>0</v>
@@ -5234,7 +5234,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>247354.82</v>
+        <v>247354.83</v>
       </c>
       <c r="F9" s="8" t="n">
         <v>2668337.97</v>
@@ -5249,7 +5249,7 @@
         <v>5222</v>
       </c>
       <c r="J9" s="9" t="n">
-        <v>242132.82</v>
+        <v>242132.83</v>
       </c>
     </row>
     <row r="10">
@@ -5259,7 +5259,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>250606.57</v>
+        <v>250606.58</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>0</v>
@@ -5268,7 +5268,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>250606.57</v>
+        <v>250606.58</v>
       </c>
       <c r="F10" s="8" t="n">
         <v>2668337.97</v>
@@ -5283,7 +5283,7 @@
         <v>5222</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>245384.57</v>
+        <v>245384.58</v>
       </c>
     </row>
     <row r="11">
@@ -5395,7 +5395,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>252440.32</v>
+        <v>252440.33</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>0</v>
@@ -5404,7 +5404,7 @@
         <v>0</v>
       </c>
       <c r="E14" s="9" t="n">
-        <v>252440.32</v>
+        <v>252440.33</v>
       </c>
       <c r="F14" s="8" t="n">
         <v>2668337.97</v>
@@ -5419,7 +5419,7 @@
         <v>5222</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>247218.32</v>
+        <v>247218.33</v>
       </c>
     </row>
     <row r="15">
@@ -5429,7 +5429,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>250364.69</v>
+        <v>250364.68</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>0</v>
@@ -5438,7 +5438,7 @@
         <v>0</v>
       </c>
       <c r="E15" s="9" t="n">
-        <v>250364.69</v>
+        <v>250364.68</v>
       </c>
       <c r="F15" s="8" t="n">
         <v>2668337.97</v>
@@ -5453,7 +5453,7 @@
         <v>5222</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>245142.69</v>
+        <v>245142.68</v>
       </c>
     </row>
     <row r="16">
@@ -5463,7 +5463,7 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>249214.31</v>
+        <v>249214.32</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>0</v>
@@ -5472,7 +5472,7 @@
         <v>0</v>
       </c>
       <c r="E16" s="9" t="n">
-        <v>249214.31</v>
+        <v>249214.32</v>
       </c>
       <c r="F16" s="8" t="n">
         <v>2668337.97</v>
@@ -5487,7 +5487,7 @@
         <v>5222</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>243992.31</v>
+        <v>243992.32</v>
       </c>
     </row>
     <row r="17">
@@ -5497,7 +5497,7 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>252592.13</v>
+        <v>252592.11</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>0</v>
@@ -5506,7 +5506,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="9" t="n">
-        <v>252592.13</v>
+        <v>252592.11</v>
       </c>
       <c r="F17" s="8" t="n">
         <v>2668337.97</v>
@@ -5521,7 +5521,7 @@
         <v>5222</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>247370.13</v>
+        <v>247370.11</v>
       </c>
     </row>
     <row r="18">
@@ -5633,7 +5633,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>255943.25</v>
+        <v>255943.24</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>0</v>
@@ -5642,7 +5642,7 @@
         <v>0</v>
       </c>
       <c r="E21" s="9" t="n">
-        <v>255943.25</v>
+        <v>255943.24</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>2668337.97</v>
@@ -5657,7 +5657,7 @@
         <v>5222</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>250721.25</v>
+        <v>250721.24</v>
       </c>
     </row>
     <row r="22">
@@ -5735,7 +5735,7 @@
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>256009.58</v>
+        <v>256009.59</v>
       </c>
       <c r="C24" s="9" t="n">
         <v>0</v>
@@ -5744,7 +5744,7 @@
         <v>0</v>
       </c>
       <c r="E24" s="9" t="n">
-        <v>256009.58</v>
+        <v>256009.59</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>2668337.97</v>
@@ -5759,7 +5759,7 @@
         <v>5222</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>250787.58</v>
+        <v>250787.59</v>
       </c>
     </row>
     <row r="25">
@@ -5803,7 +5803,7 @@
         </is>
       </c>
       <c r="B26" s="9" t="n">
-        <v>253029.42</v>
+        <v>253029.43</v>
       </c>
       <c r="C26" s="9" t="n">
         <v>0</v>
@@ -5812,7 +5812,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="9" t="n">
-        <v>253029.42</v>
+        <v>253029.43</v>
       </c>
       <c r="F26" s="8" t="n">
         <v>2668337.97</v>
@@ -5827,7 +5827,7 @@
         <v>5222</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>247807.42</v>
+        <v>247807.43</v>
       </c>
     </row>
     <row r="27">
@@ -5871,7 +5871,7 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>256918.86</v>
+        <v>256918.87</v>
       </c>
       <c r="C28" s="9" t="n">
         <v>0</v>
@@ -5880,7 +5880,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>256918.86</v>
+        <v>256918.87</v>
       </c>
       <c r="F28" s="8" t="n">
         <v>2668337.97</v>
@@ -5895,7 +5895,7 @@
         <v>5222</v>
       </c>
       <c r="J28" s="9" t="n">
-        <v>251696.86</v>
+        <v>251696.87</v>
       </c>
     </row>
     <row r="29">
@@ -5905,7 +5905,7 @@
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>259719.71</v>
+        <v>259719.72</v>
       </c>
       <c r="C29" s="9" t="n">
         <v>0</v>
@@ -5914,7 +5914,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="9" t="n">
-        <v>259719.71</v>
+        <v>259719.72</v>
       </c>
       <c r="F29" s="8" t="n">
         <v>2668337.97</v>
@@ -5929,7 +5929,7 @@
         <v>5222</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>254497.71</v>
+        <v>254497.72</v>
       </c>
     </row>
     <row r="30">
@@ -5939,7 +5939,7 @@
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>262799.85</v>
+        <v>262799.84</v>
       </c>
       <c r="C30" s="9" t="n">
         <v>0</v>
@@ -5948,7 +5948,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="9" t="n">
-        <v>262799.85</v>
+        <v>262799.84</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>2668337.97</v>
@@ -5963,7 +5963,7 @@
         <v>5222</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>257577.85</v>
+        <v>257577.84</v>
       </c>
     </row>
     <row r="31">
@@ -5973,7 +5973,7 @@
         </is>
       </c>
       <c r="B31" s="9" t="n">
-        <v>266449.95</v>
+        <v>266449.94</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>0</v>
@@ -5982,7 +5982,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="9" t="n">
-        <v>266449.95</v>
+        <v>266449.94</v>
       </c>
       <c r="F31" s="8" t="n">
         <v>2668337.97</v>
@@ -5997,7 +5997,7 @@
         <v>5222</v>
       </c>
       <c r="J31" s="9" t="n">
-        <v>261227.95</v>
+        <v>261227.94</v>
       </c>
     </row>
     <row r="32">
@@ -6007,7 +6007,7 @@
         </is>
       </c>
       <c r="B32" s="9" t="n">
-        <v>267535.21</v>
+        <v>267535.22</v>
       </c>
       <c r="C32" s="9" t="n">
         <v>0</v>
@@ -6016,7 +6016,7 @@
         <v>0</v>
       </c>
       <c r="E32" s="9" t="n">
-        <v>267535.21</v>
+        <v>267535.22</v>
       </c>
       <c r="F32" s="8" t="n">
         <v>2668337.97</v>
@@ -6031,7 +6031,7 @@
         <v>5222</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>262313.21</v>
+        <v>262313.22</v>
       </c>
     </row>
     <row r="33">
@@ -6041,7 +6041,7 @@
         </is>
       </c>
       <c r="B33" s="9" t="n">
-        <v>266846.84</v>
+        <v>266846.83</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>0</v>
@@ -6050,7 +6050,7 @@
         <v>0</v>
       </c>
       <c r="E33" s="9" t="n">
-        <v>266846.84</v>
+        <v>266846.83</v>
       </c>
       <c r="F33" s="8" t="n">
         <v>2668337.97</v>
@@ -6065,7 +6065,7 @@
         <v>5222</v>
       </c>
       <c r="J33" s="9" t="n">
-        <v>261624.84</v>
+        <v>261624.83</v>
       </c>
     </row>
     <row r="34">
@@ -6075,7 +6075,7 @@
         </is>
       </c>
       <c r="B34" s="9" t="n">
-        <v>264378.62</v>
+        <v>264378.61</v>
       </c>
       <c r="C34" s="9" t="n">
         <v>0</v>
@@ -6084,7 +6084,7 @@
         <v>0</v>
       </c>
       <c r="E34" s="9" t="n">
-        <v>264378.62</v>
+        <v>264378.61</v>
       </c>
       <c r="F34" s="8" t="n">
         <v>2668337.97</v>
@@ -6099,7 +6099,7 @@
         <v>5222</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>259156.62</v>
+        <v>259156.61</v>
       </c>
     </row>
     <row r="35">
@@ -6143,7 +6143,7 @@
         </is>
       </c>
       <c r="B36" s="9" t="n">
-        <v>264511.62</v>
+        <v>264511.61</v>
       </c>
       <c r="C36" s="9" t="n">
         <v>0</v>
@@ -6152,7 +6152,7 @@
         <v>0</v>
       </c>
       <c r="E36" s="9" t="n">
-        <v>264511.62</v>
+        <v>264511.61</v>
       </c>
       <c r="F36" s="8" t="n">
         <v>2668337.97</v>
@@ -6167,7 +6167,7 @@
         <v>5222</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>259289.62</v>
+        <v>259289.61</v>
       </c>
     </row>
     <row r="37">
@@ -6211,7 +6211,7 @@
         </is>
       </c>
       <c r="B38" s="9" t="n">
-        <v>264907.16</v>
+        <v>264907.15</v>
       </c>
       <c r="C38" s="9" t="n">
         <v>0</v>
@@ -6220,7 +6220,7 @@
         <v>0</v>
       </c>
       <c r="E38" s="9" t="n">
-        <v>264907.16</v>
+        <v>264907.15</v>
       </c>
       <c r="F38" s="8" t="n">
         <v>2668337.97</v>
@@ -6235,7 +6235,7 @@
         <v>5222</v>
       </c>
       <c r="J38" s="9" t="n">
-        <v>259685.16</v>
+        <v>259685.15</v>
       </c>
     </row>
     <row r="39">
@@ -6279,7 +6279,7 @@
         </is>
       </c>
       <c r="B40" s="9" t="n">
-        <v>262611.29</v>
+        <v>262611.27</v>
       </c>
       <c r="C40" s="9" t="n">
         <v>0</v>
@@ -6288,7 +6288,7 @@
         <v>0</v>
       </c>
       <c r="E40" s="9" t="n">
-        <v>262611.29</v>
+        <v>262611.27</v>
       </c>
       <c r="F40" s="8" t="n">
         <v>2668337.97</v>
@@ -6303,7 +6303,7 @@
         <v>5222</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>257389.29</v>
+        <v>257389.27</v>
       </c>
     </row>
     <row r="41">
@@ -6313,7 +6313,7 @@
         </is>
       </c>
       <c r="B41" s="9" t="n">
-        <v>266589.54</v>
+        <v>266589.55</v>
       </c>
       <c r="C41" s="9" t="n">
         <v>0</v>
@@ -6322,7 +6322,7 @@
         <v>0</v>
       </c>
       <c r="E41" s="9" t="n">
-        <v>266589.54</v>
+        <v>266589.55</v>
       </c>
       <c r="F41" s="8" t="n">
         <v>2668337.97</v>
@@ -6337,7 +6337,7 @@
         <v>5222</v>
       </c>
       <c r="J41" s="9" t="n">
-        <v>261367.54</v>
+        <v>261367.55</v>
       </c>
     </row>
     <row r="42">
@@ -6415,7 +6415,7 @@
         </is>
       </c>
       <c r="B44" s="9" t="n">
-        <v>227492.07</v>
+        <v>227492.08</v>
       </c>
       <c r="C44" s="9" t="n">
         <v>0</v>
@@ -6424,7 +6424,7 @@
         <v>0</v>
       </c>
       <c r="E44" s="9" t="n">
-        <v>227492.07</v>
+        <v>227492.08</v>
       </c>
       <c r="F44" s="8" t="n">
         <v>2668337.97</v>
@@ -6439,7 +6439,7 @@
         <v>5222</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>222270.07</v>
+        <v>222270.08</v>
       </c>
     </row>
     <row r="45">
@@ -6449,7 +6449,7 @@
         </is>
       </c>
       <c r="B45" s="9" t="n">
-        <v>230216.29</v>
+        <v>230216.28</v>
       </c>
       <c r="C45" s="9" t="n">
         <v>0</v>
@@ -6458,7 +6458,7 @@
         <v>0</v>
       </c>
       <c r="E45" s="9" t="n">
-        <v>230216.29</v>
+        <v>230216.28</v>
       </c>
       <c r="F45" s="8" t="n">
         <v>2668337.97</v>
@@ -6473,7 +6473,7 @@
         <v>5222</v>
       </c>
       <c r="J45" s="9" t="n">
-        <v>224994.29</v>
+        <v>224994.28</v>
       </c>
     </row>
     <row r="46">
@@ -6483,7 +6483,7 @@
         </is>
       </c>
       <c r="B46" s="9" t="n">
-        <v>227615.14</v>
+        <v>227615.13</v>
       </c>
       <c r="C46" s="9" t="n">
         <v>0</v>
@@ -6492,7 +6492,7 @@
         <v>0</v>
       </c>
       <c r="E46" s="9" t="n">
-        <v>227615.14</v>
+        <v>227615.13</v>
       </c>
       <c r="F46" s="8" t="n">
         <v>2668337.97</v>
@@ -6507,7 +6507,7 @@
         <v>5222</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>222393.14</v>
+        <v>222393.13</v>
       </c>
     </row>
     <row r="47">
@@ -6585,7 +6585,7 @@
         </is>
       </c>
       <c r="B49" s="9" t="n">
-        <v>243638.95</v>
+        <v>243638.93</v>
       </c>
       <c r="C49" s="9" t="n">
         <v>0</v>
@@ -6594,7 +6594,7 @@
         <v>0</v>
       </c>
       <c r="E49" s="9" t="n">
-        <v>243638.95</v>
+        <v>243638.93</v>
       </c>
       <c r="F49" s="8" t="n">
         <v>2668337.97</v>
@@ -6609,7 +6609,7 @@
         <v>5222</v>
       </c>
       <c r="J49" s="9" t="n">
-        <v>238416.95</v>
+        <v>238416.93</v>
       </c>
     </row>
     <row r="50">
@@ -6789,7 +6789,7 @@
         </is>
       </c>
       <c r="B55" s="9" t="n">
-        <v>253596.44</v>
+        <v>253596.41</v>
       </c>
       <c r="C55" s="9" t="n">
         <v>0</v>
@@ -6798,7 +6798,7 @@
         <v>0</v>
       </c>
       <c r="E55" s="9" t="n">
-        <v>253596.44</v>
+        <v>253596.41</v>
       </c>
       <c r="F55" s="8" t="n">
         <v>2668337.97</v>
@@ -6813,7 +6813,7 @@
         <v>5222</v>
       </c>
       <c r="J55" s="9" t="n">
-        <v>248374.44</v>
+        <v>248374.41</v>
       </c>
     </row>
     <row r="56">
@@ -6823,7 +6823,7 @@
         </is>
       </c>
       <c r="B56" s="9" t="n">
-        <v>253244.21</v>
+        <v>253244.22</v>
       </c>
       <c r="C56" s="9" t="n">
         <v>0</v>
@@ -6832,7 +6832,7 @@
         <v>0</v>
       </c>
       <c r="E56" s="9" t="n">
-        <v>253244.21</v>
+        <v>253244.22</v>
       </c>
       <c r="F56" s="8" t="n">
         <v>2668337.97</v>
@@ -6847,7 +6847,7 @@
         <v>5222</v>
       </c>
       <c r="J56" s="9" t="n">
-        <v>248022.21</v>
+        <v>248022.22</v>
       </c>
     </row>
     <row r="57">
@@ -6857,7 +6857,7 @@
         </is>
       </c>
       <c r="B57" s="9" t="n">
-        <v>254946.35</v>
+        <v>254946.34</v>
       </c>
       <c r="C57" s="9" t="n">
         <v>0</v>
@@ -6866,7 +6866,7 @@
         <v>0</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>254946.35</v>
+        <v>254946.34</v>
       </c>
       <c r="F57" s="8" t="n">
         <v>2668337.97</v>
@@ -6881,7 +6881,7 @@
         <v>5222</v>
       </c>
       <c r="J57" s="9" t="n">
-        <v>249724.35</v>
+        <v>249724.34</v>
       </c>
     </row>
     <row r="58">
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="B58" s="9" t="n">
-        <v>256210.35</v>
+        <v>256210.34</v>
       </c>
       <c r="C58" s="9" t="n">
         <v>0</v>
@@ -6900,7 +6900,7 @@
         <v>0</v>
       </c>
       <c r="E58" s="9" t="n">
-        <v>256210.35</v>
+        <v>256210.34</v>
       </c>
       <c r="F58" s="8" t="n">
         <v>2668337.97</v>
@@ -6915,7 +6915,7 @@
         <v>5222</v>
       </c>
       <c r="J58" s="9" t="n">
-        <v>250988.35</v>
+        <v>250988.34</v>
       </c>
     </row>
     <row r="59">
@@ -6925,7 +6925,7 @@
         </is>
       </c>
       <c r="B59" s="9" t="n">
-        <v>255603.99</v>
+        <v>255603.98</v>
       </c>
       <c r="C59" s="9" t="n">
         <v>0</v>
@@ -6934,7 +6934,7 @@
         <v>0</v>
       </c>
       <c r="E59" s="9" t="n">
-        <v>255603.99</v>
+        <v>255603.98</v>
       </c>
       <c r="F59" s="8" t="n">
         <v>2668337.97</v>
@@ -6949,7 +6949,7 @@
         <v>5222</v>
       </c>
       <c r="J59" s="9" t="n">
-        <v>250381.99</v>
+        <v>250381.98</v>
       </c>
     </row>
     <row r="60">
@@ -6959,7 +6959,7 @@
         </is>
       </c>
       <c r="B60" s="9" t="n">
-        <v>253917.16</v>
+        <v>253917.15</v>
       </c>
       <c r="C60" s="9" t="n">
         <v>0</v>
@@ -6968,7 +6968,7 @@
         <v>0</v>
       </c>
       <c r="E60" s="9" t="n">
-        <v>253917.16</v>
+        <v>253917.15</v>
       </c>
       <c r="F60" s="8" t="n">
         <v>2668337.97</v>
@@ -6983,7 +6983,7 @@
         <v>5222</v>
       </c>
       <c r="J60" s="9" t="n">
-        <v>248695.16</v>
+        <v>248695.15</v>
       </c>
     </row>
     <row r="61">
@@ -6993,7 +6993,7 @@
         </is>
       </c>
       <c r="B61" s="9" t="n">
-        <v>255005.43</v>
+        <v>255005.41</v>
       </c>
       <c r="C61" s="9" t="n">
         <v>0</v>
@@ -7002,7 +7002,7 @@
         <v>0</v>
       </c>
       <c r="E61" s="9" t="n">
-        <v>255005.43</v>
+        <v>255005.41</v>
       </c>
       <c r="F61" s="8" t="n">
         <v>2668337.97</v>
@@ -7017,7 +7017,7 @@
         <v>5222</v>
       </c>
       <c r="J61" s="9" t="n">
-        <v>249783.43</v>
+        <v>249783.41</v>
       </c>
     </row>
     <row r="62">
@@ -7197,7 +7197,7 @@
         </is>
       </c>
       <c r="B67" s="9" t="n">
-        <v>270728.3</v>
+        <v>270728.31</v>
       </c>
       <c r="C67" s="9" t="n">
         <v>0</v>
@@ -7206,7 +7206,7 @@
         <v>0</v>
       </c>
       <c r="E67" s="9" t="n">
-        <v>270728.3</v>
+        <v>270728.31</v>
       </c>
       <c r="F67" s="8" t="n">
         <v>2668337.97</v>
@@ -7221,7 +7221,7 @@
         <v>5222</v>
       </c>
       <c r="J67" s="9" t="n">
-        <v>265506.3</v>
+        <v>265506.31</v>
       </c>
     </row>
     <row r="68">
@@ -7231,7 +7231,7 @@
         </is>
       </c>
       <c r="B68" s="9" t="n">
-        <v>269402.99</v>
+        <v>269403</v>
       </c>
       <c r="C68" s="9" t="n">
         <v>0</v>
@@ -7240,7 +7240,7 @@
         <v>0</v>
       </c>
       <c r="E68" s="9" t="n">
-        <v>269402.99</v>
+        <v>269403</v>
       </c>
       <c r="F68" s="8" t="n">
         <v>2668337.97</v>
@@ -7255,7 +7255,7 @@
         <v>5222</v>
       </c>
       <c r="J68" s="9" t="n">
-        <v>264180.99</v>
+        <v>264181</v>
       </c>
     </row>
     <row r="69">
@@ -7333,7 +7333,7 @@
         </is>
       </c>
       <c r="B71" s="9" t="n">
-        <v>271985.32</v>
+        <v>271985.31</v>
       </c>
       <c r="C71" s="9" t="n">
         <v>0</v>
@@ -7342,7 +7342,7 @@
         <v>0</v>
       </c>
       <c r="E71" s="9" t="n">
-        <v>271985.32</v>
+        <v>271985.31</v>
       </c>
       <c r="F71" s="8" t="n">
         <v>2668337.97</v>
@@ -7357,7 +7357,7 @@
         <v>5222</v>
       </c>
       <c r="J71" s="9" t="n">
-        <v>266763.32</v>
+        <v>266763.31</v>
       </c>
     </row>
     <row r="72">
@@ -7367,7 +7367,7 @@
         </is>
       </c>
       <c r="B72" s="9" t="n">
-        <v>273827.65</v>
+        <v>273827.66</v>
       </c>
       <c r="C72" s="9" t="n">
         <v>0</v>
@@ -7376,7 +7376,7 @@
         <v>0</v>
       </c>
       <c r="E72" s="9" t="n">
-        <v>273827.65</v>
+        <v>273827.66</v>
       </c>
       <c r="F72" s="8" t="n">
         <v>2668337.97</v>
@@ -7391,7 +7391,7 @@
         <v>5222</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>268605.65</v>
+        <v>268605.66</v>
       </c>
     </row>
     <row r="73">
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="B73" s="9" t="n">
-        <v>275223.08</v>
+        <v>275223.07</v>
       </c>
       <c r="C73" s="9" t="n">
         <v>0</v>
@@ -7410,7 +7410,7 @@
         <v>0</v>
       </c>
       <c r="E73" s="9" t="n">
-        <v>275223.08</v>
+        <v>275223.07</v>
       </c>
       <c r="F73" s="8" t="n">
         <v>2668337.97</v>
@@ -7425,7 +7425,7 @@
         <v>5222</v>
       </c>
       <c r="J73" s="9" t="n">
-        <v>270001.08</v>
+        <v>270001.07</v>
       </c>
     </row>
     <row r="74">
@@ -7435,7 +7435,7 @@
         </is>
       </c>
       <c r="B74" s="9" t="n">
-        <v>276364.36</v>
+        <v>276364.37</v>
       </c>
       <c r="C74" s="9" t="n">
         <v>0</v>
@@ -7444,7 +7444,7 @@
         <v>0</v>
       </c>
       <c r="E74" s="9" t="n">
-        <v>276364.36</v>
+        <v>276364.37</v>
       </c>
       <c r="F74" s="8" t="n">
         <v>2668337.97</v>
@@ -7459,7 +7459,7 @@
         <v>5222</v>
       </c>
       <c r="J74" s="9" t="n">
-        <v>271142.36</v>
+        <v>271142.37</v>
       </c>
     </row>
     <row r="75">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="B77" s="9" t="n">
-        <v>274905.36</v>
+        <v>274905.35</v>
       </c>
       <c r="C77" s="9" t="n">
         <v>0</v>
@@ -7546,7 +7546,7 @@
         <v>0</v>
       </c>
       <c r="E77" s="9" t="n">
-        <v>274905.36</v>
+        <v>274905.35</v>
       </c>
       <c r="F77" s="8" t="n">
         <v>2668337.97</v>
@@ -7561,7 +7561,7 @@
         <v>5222</v>
       </c>
       <c r="J77" s="9" t="n">
-        <v>269683.36</v>
+        <v>269683.35</v>
       </c>
     </row>
     <row r="78">
@@ -7571,7 +7571,7 @@
         </is>
       </c>
       <c r="B78" s="9" t="n">
-        <v>277017.4</v>
+        <v>277017.39</v>
       </c>
       <c r="C78" s="9" t="n">
         <v>0</v>
@@ -7580,7 +7580,7 @@
         <v>0</v>
       </c>
       <c r="E78" s="9" t="n">
-        <v>277017.4</v>
+        <v>277017.39</v>
       </c>
       <c r="F78" s="8" t="n">
         <v>2668337.97</v>
@@ -7595,7 +7595,7 @@
         <v>5222</v>
       </c>
       <c r="J78" s="9" t="n">
-        <v>271795.4</v>
+        <v>271795.39</v>
       </c>
     </row>
     <row r="79">
@@ -7673,7 +7673,7 @@
         </is>
       </c>
       <c r="B81" s="9" t="n">
-        <v>281999.08</v>
+        <v>281999.1</v>
       </c>
       <c r="C81" s="9" t="n">
         <v>0</v>
@@ -7682,7 +7682,7 @@
         <v>0</v>
       </c>
       <c r="E81" s="9" t="n">
-        <v>281999.08</v>
+        <v>281999.1</v>
       </c>
       <c r="F81" s="8" t="n">
         <v>2668337.97</v>
@@ -7697,7 +7697,7 @@
         <v>5222</v>
       </c>
       <c r="J81" s="9" t="n">
-        <v>276777.08</v>
+        <v>276777.1</v>
       </c>
     </row>
     <row r="82">
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="B83" s="9" t="n">
-        <v>284275.44</v>
+        <v>284275.43</v>
       </c>
       <c r="C83" s="9" t="n">
         <v>0</v>
@@ -7750,7 +7750,7 @@
         <v>0</v>
       </c>
       <c r="E83" s="9" t="n">
-        <v>284275.44</v>
+        <v>284275.43</v>
       </c>
       <c r="F83" s="8" t="n">
         <v>2668337.97</v>
@@ -7765,7 +7765,7 @@
         <v>5222</v>
       </c>
       <c r="J83" s="9" t="n">
-        <v>279053.44</v>
+        <v>279053.43</v>
       </c>
     </row>
     <row r="84">
@@ -7775,7 +7775,7 @@
         </is>
       </c>
       <c r="B84" s="9" t="n">
-        <v>285022.54</v>
+        <v>285022.53</v>
       </c>
       <c r="C84" s="9" t="n">
         <v>0</v>
@@ -7784,7 +7784,7 @@
         <v>0</v>
       </c>
       <c r="E84" s="9" t="n">
-        <v>285022.54</v>
+        <v>285022.53</v>
       </c>
       <c r="F84" s="8" t="n">
         <v>2668337.97</v>
@@ -7799,7 +7799,7 @@
         <v>5222</v>
       </c>
       <c r="J84" s="9" t="n">
-        <v>279800.54</v>
+        <v>279800.53</v>
       </c>
     </row>
     <row r="85">
@@ -7809,7 +7809,7 @@
         </is>
       </c>
       <c r="B85" s="9" t="n">
-        <v>286673.49</v>
+        <v>286673.48</v>
       </c>
       <c r="C85" s="9" t="n">
         <v>0</v>
@@ -7818,7 +7818,7 @@
         <v>0</v>
       </c>
       <c r="E85" s="9" t="n">
-        <v>286673.49</v>
+        <v>286673.48</v>
       </c>
       <c r="F85" s="8" t="n">
         <v>2668337.97</v>
@@ -7833,7 +7833,7 @@
         <v>5222</v>
       </c>
       <c r="J85" s="9" t="n">
-        <v>281451.49</v>
+        <v>281451.48</v>
       </c>
     </row>
     <row r="86">
@@ -7911,7 +7911,7 @@
         </is>
       </c>
       <c r="B88" s="9" t="n">
-        <v>289294.52</v>
+        <v>289294.53</v>
       </c>
       <c r="C88" s="9" t="n">
         <v>0</v>
@@ -7920,7 +7920,7 @@
         <v>0</v>
       </c>
       <c r="E88" s="9" t="n">
-        <v>289294.52</v>
+        <v>289294.53</v>
       </c>
       <c r="F88" s="8" t="n">
         <v>2668337.97</v>
@@ -7935,7 +7935,7 @@
         <v>5222</v>
       </c>
       <c r="J88" s="9" t="n">
-        <v>284072.52</v>
+        <v>284072.53</v>
       </c>
     </row>
     <row r="89">
@@ -7945,7 +7945,7 @@
         </is>
       </c>
       <c r="B89" s="9" t="n">
-        <v>292009.84</v>
+        <v>292009.83</v>
       </c>
       <c r="C89" s="9" t="n">
         <v>0</v>
@@ -7954,7 +7954,7 @@
         <v>0</v>
       </c>
       <c r="E89" s="9" t="n">
-        <v>292009.84</v>
+        <v>292009.83</v>
       </c>
       <c r="F89" s="8" t="n">
         <v>2668337.97</v>
@@ -7969,7 +7969,7 @@
         <v>5222</v>
       </c>
       <c r="J89" s="9" t="n">
-        <v>286787.84</v>
+        <v>286787.83</v>
       </c>
     </row>
     <row r="90">
@@ -7979,7 +7979,7 @@
         </is>
       </c>
       <c r="B90" s="9" t="n">
-        <v>293317.69</v>
+        <v>293317.7</v>
       </c>
       <c r="C90" s="9" t="n">
         <v>0</v>
@@ -7988,7 +7988,7 @@
         <v>0</v>
       </c>
       <c r="E90" s="9" t="n">
-        <v>293317.69</v>
+        <v>293317.7</v>
       </c>
       <c r="F90" s="8" t="n">
         <v>2668337.97</v>
@@ -8003,7 +8003,7 @@
         <v>5222</v>
       </c>
       <c r="J90" s="9" t="n">
-        <v>288095.69</v>
+        <v>288095.7</v>
       </c>
     </row>
     <row r="91">
@@ -8013,7 +8013,7 @@
         </is>
       </c>
       <c r="B91" s="9" t="n">
-        <v>292026.71</v>
+        <v>292026.72</v>
       </c>
       <c r="C91" s="9" t="n">
         <v>0</v>
@@ -8022,7 +8022,7 @@
         <v>0</v>
       </c>
       <c r="E91" s="9" t="n">
-        <v>292026.71</v>
+        <v>292026.72</v>
       </c>
       <c r="F91" s="8" t="n">
         <v>2668337.97</v>
@@ -8037,7 +8037,7 @@
         <v>5222</v>
       </c>
       <c r="J91" s="9" t="n">
-        <v>286804.71</v>
+        <v>286804.72</v>
       </c>
     </row>
     <row r="92">
@@ -8047,7 +8047,7 @@
         </is>
       </c>
       <c r="B92" s="9" t="n">
-        <v>432786.25</v>
+        <v>432786.24</v>
       </c>
       <c r="C92" s="9" t="n">
         <v>0</v>
@@ -8056,7 +8056,7 @@
         <v>0</v>
       </c>
       <c r="E92" s="9" t="n">
-        <v>432786.25</v>
+        <v>432786.24</v>
       </c>
       <c r="F92" s="8" t="n">
         <v>3897262.79</v>
@@ -8071,7 +8071,7 @@
         <v>122222</v>
       </c>
       <c r="J92" s="9" t="n">
-        <v>310564.25</v>
+        <v>310564.24</v>
       </c>
     </row>
     <row r="93">
@@ -8183,7 +8183,7 @@
         </is>
       </c>
       <c r="B96" s="9" t="n">
-        <v>437052.21</v>
+        <v>437052.22</v>
       </c>
       <c r="C96" s="9" t="n">
         <v>0</v>
@@ -8192,7 +8192,7 @@
         <v>0</v>
       </c>
       <c r="E96" s="9" t="n">
-        <v>437052.21</v>
+        <v>437052.22</v>
       </c>
       <c r="F96" s="8" t="n">
         <v>3897262.79</v>
@@ -8207,7 +8207,7 @@
         <v>11052</v>
       </c>
       <c r="J96" s="9" t="n">
-        <v>426000.21</v>
+        <v>426000.22</v>
       </c>
     </row>
     <row r="97">
@@ -8251,7 +8251,7 @@
         </is>
       </c>
       <c r="B98" s="9" t="n">
-        <v>440268.39</v>
+        <v>440268.4</v>
       </c>
       <c r="C98" s="9" t="n">
         <v>0</v>
@@ -8260,7 +8260,7 @@
         <v>0</v>
       </c>
       <c r="E98" s="9" t="n">
-        <v>440268.39</v>
+        <v>440268.4</v>
       </c>
       <c r="F98" s="8" t="n">
         <v>3897262.79</v>
@@ -8275,7 +8275,7 @@
         <v>11052</v>
       </c>
       <c r="J98" s="9" t="n">
-        <v>429216.39</v>
+        <v>429216.4</v>
       </c>
     </row>
     <row r="99">
@@ -8353,7 +8353,7 @@
         </is>
       </c>
       <c r="B101" s="9" t="n">
-        <v>435849.11</v>
+        <v>435849.09</v>
       </c>
       <c r="C101" s="9" t="n">
         <v>0</v>
@@ -8362,7 +8362,7 @@
         <v>0</v>
       </c>
       <c r="E101" s="9" t="n">
-        <v>435849.11</v>
+        <v>435849.09</v>
       </c>
       <c r="F101" s="8" t="n">
         <v>3897262.79</v>
@@ -8377,7 +8377,7 @@
         <v>11052</v>
       </c>
       <c r="J101" s="9" t="n">
-        <v>424797.11</v>
+        <v>424797.09</v>
       </c>
     </row>
     <row r="102">
@@ -8387,7 +8387,7 @@
         </is>
       </c>
       <c r="B102" s="9" t="n">
-        <v>435994.31</v>
+        <v>435994.3</v>
       </c>
       <c r="C102" s="9" t="n">
         <v>0</v>
@@ -8396,7 +8396,7 @@
         <v>0</v>
       </c>
       <c r="E102" s="9" t="n">
-        <v>435994.31</v>
+        <v>435994.3</v>
       </c>
       <c r="F102" s="8" t="n">
         <v>3897262.79</v>
@@ -8411,7 +8411,7 @@
         <v>11052</v>
       </c>
       <c r="J102" s="9" t="n">
-        <v>424942.31</v>
+        <v>424942.3</v>
       </c>
     </row>
     <row r="103">
@@ -8455,7 +8455,7 @@
         </is>
       </c>
       <c r="B104" s="9" t="n">
-        <v>437774.31</v>
+        <v>437774.29</v>
       </c>
       <c r="C104" s="9" t="n">
         <v>0</v>
@@ -8464,7 +8464,7 @@
         <v>0</v>
       </c>
       <c r="E104" s="9" t="n">
-        <v>437774.31</v>
+        <v>437774.29</v>
       </c>
       <c r="F104" s="8" t="n">
         <v>3897262.79</v>
@@ -8479,7 +8479,7 @@
         <v>11052</v>
       </c>
       <c r="J104" s="9" t="n">
-        <v>426722.31</v>
+        <v>426722.29</v>
       </c>
     </row>
     <row r="105">
@@ -8489,7 +8489,7 @@
         </is>
       </c>
       <c r="B105" s="9" t="n">
-        <v>439437.01</v>
+        <v>439437.02</v>
       </c>
       <c r="C105" s="9" t="n">
         <v>0</v>
@@ -8498,7 +8498,7 @@
         <v>0</v>
       </c>
       <c r="E105" s="9" t="n">
-        <v>439437.01</v>
+        <v>439437.02</v>
       </c>
       <c r="F105" s="8" t="n">
         <v>3897262.79</v>
@@ -8513,7 +8513,7 @@
         <v>11052</v>
       </c>
       <c r="J105" s="9" t="n">
-        <v>428385.01</v>
+        <v>428385.02</v>
       </c>
     </row>
     <row r="106">
@@ -8523,7 +8523,7 @@
         </is>
       </c>
       <c r="B106" s="9" t="n">
-        <v>436300.23</v>
+        <v>436300.22</v>
       </c>
       <c r="C106" s="9" t="n">
         <v>0</v>
@@ -8532,7 +8532,7 @@
         <v>0</v>
       </c>
       <c r="E106" s="9" t="n">
-        <v>436300.23</v>
+        <v>436300.22</v>
       </c>
       <c r="F106" s="8" t="n">
         <v>3897262.79</v>
@@ -8547,7 +8547,7 @@
         <v>11052</v>
       </c>
       <c r="J106" s="9" t="n">
-        <v>425248.23</v>
+        <v>425248.22</v>
       </c>
     </row>
     <row r="107">
@@ -8557,7 +8557,7 @@
         </is>
       </c>
       <c r="B107" s="9" t="n">
-        <v>441510.35</v>
+        <v>441510.36</v>
       </c>
       <c r="C107" s="9" t="n">
         <v>0</v>
@@ -8566,7 +8566,7 @@
         <v>0</v>
       </c>
       <c r="E107" s="9" t="n">
-        <v>441510.35</v>
+        <v>441510.36</v>
       </c>
       <c r="F107" s="8" t="n">
         <v>3897262.79</v>
@@ -8581,7 +8581,7 @@
         <v>11052</v>
       </c>
       <c r="J107" s="9" t="n">
-        <v>430458.35</v>
+        <v>430458.36</v>
       </c>
     </row>
     <row r="108">
@@ -8591,7 +8591,7 @@
         </is>
       </c>
       <c r="B108" s="9" t="n">
-        <v>427803.72</v>
+        <v>427803.74</v>
       </c>
       <c r="C108" s="9" t="n">
         <v>0</v>
@@ -8600,7 +8600,7 @@
         <v>0</v>
       </c>
       <c r="E108" s="9" t="n">
-        <v>427803.72</v>
+        <v>427803.74</v>
       </c>
       <c r="F108" s="8" t="n">
         <v>3897262.79</v>
@@ -8615,7 +8615,7 @@
         <v>-307408</v>
       </c>
       <c r="J108" s="9" t="n">
-        <v>735211.72</v>
+        <v>735211.74</v>
       </c>
     </row>
     <row r="109">
@@ -8625,7 +8625,7 @@
         </is>
       </c>
       <c r="B109" s="9" t="n">
-        <v>432917.69</v>
+        <v>432917.68</v>
       </c>
       <c r="C109" s="9" t="n">
         <v>0</v>
@@ -8634,7 +8634,7 @@
         <v>0</v>
       </c>
       <c r="E109" s="9" t="n">
-        <v>432917.69</v>
+        <v>432917.68</v>
       </c>
       <c r="F109" s="8" t="n">
         <v>3897262.79</v>
@@ -8649,7 +8649,7 @@
         <v>-307408</v>
       </c>
       <c r="J109" s="9" t="n">
-        <v>740325.6899999999</v>
+        <v>740325.6800000001</v>
       </c>
     </row>
     <row r="110">
@@ -8659,7 +8659,7 @@
         </is>
       </c>
       <c r="B110" s="9" t="n">
-        <v>435630.96</v>
+        <v>435630.98</v>
       </c>
       <c r="C110" s="9" t="n">
         <v>0</v>
@@ -8668,7 +8668,7 @@
         <v>0</v>
       </c>
       <c r="E110" s="9" t="n">
-        <v>435630.96</v>
+        <v>435630.98</v>
       </c>
       <c r="F110" s="8" t="n">
         <v>3897262.79</v>
@@ -8683,7 +8683,7 @@
         <v>-385208</v>
       </c>
       <c r="J110" s="9" t="n">
-        <v>820838.96</v>
+        <v>820838.98</v>
       </c>
     </row>
     <row r="111">
@@ -8693,7 +8693,7 @@
         </is>
       </c>
       <c r="B111" s="9" t="n">
-        <v>432862.76</v>
+        <v>432862.77</v>
       </c>
       <c r="C111" s="9" t="n">
         <v>0</v>
@@ -8702,7 +8702,7 @@
         <v>0</v>
       </c>
       <c r="E111" s="9" t="n">
-        <v>432862.76</v>
+        <v>432862.77</v>
       </c>
       <c r="F111" s="8" t="n">
         <v>3897262.79</v>
@@ -8717,7 +8717,7 @@
         <v>-385208</v>
       </c>
       <c r="J111" s="9" t="n">
-        <v>818070.76</v>
+        <v>818070.77</v>
       </c>
     </row>
     <row r="112">
@@ -8727,7 +8727,7 @@
         </is>
       </c>
       <c r="B112" s="9" t="n">
-        <v>430768.43</v>
+        <v>430768.44</v>
       </c>
       <c r="C112" s="9" t="n">
         <v>0</v>
@@ -8736,7 +8736,7 @@
         <v>0</v>
       </c>
       <c r="E112" s="9" t="n">
-        <v>430768.43</v>
+        <v>430768.44</v>
       </c>
       <c r="F112" s="8" t="n">
         <v>3897262.79</v>
@@ -8751,7 +8751,7 @@
         <v>-385208</v>
       </c>
       <c r="J112" s="9" t="n">
-        <v>815976.4300000001</v>
+        <v>815976.4399999999</v>
       </c>
     </row>
     <row r="113">
@@ -8795,7 +8795,7 @@
         </is>
       </c>
       <c r="B114" s="9" t="n">
-        <v>442100.61</v>
+        <v>442100.59</v>
       </c>
       <c r="C114" s="9" t="n">
         <v>0</v>
@@ -8804,7 +8804,7 @@
         <v>0</v>
       </c>
       <c r="E114" s="9" t="n">
-        <v>442100.61</v>
+        <v>442100.59</v>
       </c>
       <c r="F114" s="8" t="n">
         <v>3897262.79</v>
@@ -8819,7 +8819,7 @@
         <v>-385208</v>
       </c>
       <c r="J114" s="9" t="n">
-        <v>827308.61</v>
+        <v>827308.59</v>
       </c>
     </row>
     <row r="115">
@@ -8863,7 +8863,7 @@
         </is>
       </c>
       <c r="B116" s="9" t="n">
-        <v>456359.72</v>
+        <v>456359.73</v>
       </c>
       <c r="C116" s="9" t="n">
         <v>0</v>
@@ -8872,7 +8872,7 @@
         <v>0</v>
       </c>
       <c r="E116" s="9" t="n">
-        <v>456359.72</v>
+        <v>456359.73</v>
       </c>
       <c r="F116" s="8" t="n">
         <v>3897262.79</v>
@@ -8887,7 +8887,7 @@
         <v>-401434</v>
       </c>
       <c r="J116" s="9" t="n">
-        <v>857793.72</v>
+        <v>857793.73</v>
       </c>
     </row>
     <row r="117">
@@ -8931,7 +8931,7 @@
         </is>
       </c>
       <c r="B118" s="9" t="n">
-        <v>458121.09</v>
+        <v>458121.11</v>
       </c>
       <c r="C118" s="9" t="n">
         <v>0</v>
@@ -8940,7 +8940,7 @@
         <v>0</v>
       </c>
       <c r="E118" s="9" t="n">
-        <v>458121.09</v>
+        <v>458121.11</v>
       </c>
       <c r="F118" s="8" t="n">
         <v>3897262.79</v>
@@ -8955,7 +8955,7 @@
         <v>-504674</v>
       </c>
       <c r="J118" s="9" t="n">
-        <v>962795.09</v>
+        <v>962795.11</v>
       </c>
     </row>
     <row r="119">
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="B119" s="9" t="n">
-        <v>459377.75</v>
+        <v>459377.76</v>
       </c>
       <c r="C119" s="9" t="n">
         <v>0</v>
@@ -8974,7 +8974,7 @@
         <v>0</v>
       </c>
       <c r="E119" s="9" t="n">
-        <v>459377.75</v>
+        <v>459377.76</v>
       </c>
       <c r="F119" s="8" t="n">
         <v>3897262.79</v>
@@ -8989,7 +8989,7 @@
         <v>-504674</v>
       </c>
       <c r="J119" s="9" t="n">
-        <v>964051.75</v>
+        <v>964051.76</v>
       </c>
     </row>
     <row r="120">
@@ -8999,7 +8999,7 @@
         </is>
       </c>
       <c r="B120" s="9" t="n">
-        <v>453947.08</v>
+        <v>453947.07</v>
       </c>
       <c r="C120" s="9" t="n">
         <v>0</v>
@@ -9008,7 +9008,7 @@
         <v>0</v>
       </c>
       <c r="E120" s="9" t="n">
-        <v>453947.08</v>
+        <v>453947.07</v>
       </c>
       <c r="F120" s="8" t="n">
         <v>3897262.79</v>
@@ -9023,7 +9023,7 @@
         <v>-504674</v>
       </c>
       <c r="J120" s="9" t="n">
-        <v>958621.08</v>
+        <v>958621.0699999999</v>
       </c>
     </row>
     <row r="121">
@@ -9033,7 +9033,7 @@
         </is>
       </c>
       <c r="B121" s="9" t="n">
-        <v>438010.72</v>
+        <v>438010.74</v>
       </c>
       <c r="C121" s="9" t="n">
         <v>0</v>
@@ -9042,7 +9042,7 @@
         <v>0</v>
       </c>
       <c r="E121" s="9" t="n">
-        <v>438010.72</v>
+        <v>438010.74</v>
       </c>
       <c r="F121" s="8" t="n">
         <v>3897262.79</v>
@@ -9057,7 +9057,7 @@
         <v>-504674</v>
       </c>
       <c r="J121" s="9" t="n">
-        <v>942684.72</v>
+        <v>942684.74</v>
       </c>
     </row>
     <row r="122">
@@ -9067,7 +9067,7 @@
         </is>
       </c>
       <c r="B122" s="9" t="n">
-        <v>430870.83</v>
+        <v>430870.84</v>
       </c>
       <c r="C122" s="9" t="n">
         <v>0</v>
@@ -9076,7 +9076,7 @@
         <v>0</v>
       </c>
       <c r="E122" s="9" t="n">
-        <v>430870.83</v>
+        <v>430870.84</v>
       </c>
       <c r="F122" s="8" t="n">
         <v>3897262.79</v>
@@ -9091,7 +9091,7 @@
         <v>-504674</v>
       </c>
       <c r="J122" s="9" t="n">
-        <v>935544.83</v>
+        <v>935544.84</v>
       </c>
     </row>
     <row r="123">
@@ -9101,7 +9101,7 @@
         </is>
       </c>
       <c r="B123" s="9" t="n">
-        <v>422687.32</v>
+        <v>422687.29</v>
       </c>
       <c r="C123" s="9" t="n">
         <v>0</v>
@@ -9110,7 +9110,7 @@
         <v>0</v>
       </c>
       <c r="E123" s="9" t="n">
-        <v>422687.32</v>
+        <v>422687.29</v>
       </c>
       <c r="F123" s="8" t="n">
         <v>3897262.79</v>
@@ -9125,7 +9125,7 @@
         <v>-504674</v>
       </c>
       <c r="J123" s="9" t="n">
-        <v>927361.3199999999</v>
+        <v>927361.29</v>
       </c>
     </row>
     <row r="124">
@@ -9135,7 +9135,7 @@
         </is>
       </c>
       <c r="B124" s="9" t="n">
-        <v>434850.94</v>
+        <v>434850.95</v>
       </c>
       <c r="C124" s="9" t="n">
         <v>0</v>
@@ -9144,7 +9144,7 @@
         <v>0</v>
       </c>
       <c r="E124" s="9" t="n">
-        <v>434850.94</v>
+        <v>434850.95</v>
       </c>
       <c r="F124" s="8" t="n">
         <v>3897262.79</v>
@@ -9159,7 +9159,7 @@
         <v>-263014</v>
       </c>
       <c r="J124" s="9" t="n">
-        <v>697864.9399999999</v>
+        <v>697864.95</v>
       </c>
     </row>
     <row r="125">
@@ -9203,7 +9203,7 @@
         </is>
       </c>
       <c r="B126" s="9" t="n">
-        <v>447512.26</v>
+        <v>447512.25</v>
       </c>
       <c r="C126" s="9" t="n">
         <v>0</v>
@@ -9212,7 +9212,7 @@
         <v>0</v>
       </c>
       <c r="E126" s="9" t="n">
-        <v>447512.26</v>
+        <v>447512.25</v>
       </c>
       <c r="F126" s="8" t="n">
         <v>3897262.79</v>
@@ -9227,7 +9227,7 @@
         <v>-258114</v>
       </c>
       <c r="J126" s="9" t="n">
-        <v>705626.26</v>
+        <v>705626.25</v>
       </c>
     </row>
     <row r="127">
@@ -9237,7 +9237,7 @@
         </is>
       </c>
       <c r="B127" s="9" t="n">
-        <v>453194.14</v>
+        <v>453194.12</v>
       </c>
       <c r="C127" s="9" t="n">
         <v>0</v>
@@ -9246,7 +9246,7 @@
         <v>0</v>
       </c>
       <c r="E127" s="9" t="n">
-        <v>453194.14</v>
+        <v>453194.12</v>
       </c>
       <c r="F127" s="8" t="n">
         <v>3897262.79</v>
@@ -9261,7 +9261,7 @@
         <v>-373564</v>
       </c>
       <c r="J127" s="9" t="n">
-        <v>826758.14</v>
+        <v>826758.12</v>
       </c>
     </row>
     <row r="128">
@@ -9271,7 +9271,7 @@
         </is>
       </c>
       <c r="B128" s="9" t="n">
-        <v>449942.61</v>
+        <v>449942.59</v>
       </c>
       <c r="C128" s="9" t="n">
         <v>0</v>
@@ -9280,7 +9280,7 @@
         <v>0</v>
       </c>
       <c r="E128" s="9" t="n">
-        <v>449942.61</v>
+        <v>449942.59</v>
       </c>
       <c r="F128" s="8" t="n">
         <v>3897262.79</v>
@@ -9295,7 +9295,7 @@
         <v>-373564</v>
       </c>
       <c r="J128" s="9" t="n">
-        <v>823506.61</v>
+        <v>823506.59</v>
       </c>
     </row>
     <row r="129">
@@ -9305,7 +9305,7 @@
         </is>
       </c>
       <c r="B129" s="9" t="n">
-        <v>456715.43</v>
+        <v>456715.46</v>
       </c>
       <c r="C129" s="9" t="n">
         <v>0</v>
@@ -9314,7 +9314,7 @@
         <v>0</v>
       </c>
       <c r="E129" s="9" t="n">
-        <v>456715.43</v>
+        <v>456715.46</v>
       </c>
       <c r="F129" s="8" t="n">
         <v>3897262.79</v>
@@ -9329,7 +9329,7 @@
         <v>-373564</v>
       </c>
       <c r="J129" s="9" t="n">
-        <v>830279.4300000001</v>
+        <v>830279.46</v>
       </c>
     </row>
     <row r="130">
@@ -9339,7 +9339,7 @@
         </is>
       </c>
       <c r="B130" s="9" t="n">
-        <v>460499.96</v>
+        <v>460499.93</v>
       </c>
       <c r="C130" s="9" t="n">
         <v>0</v>
@@ -9348,7 +9348,7 @@
         <v>0</v>
       </c>
       <c r="E130" s="9" t="n">
-        <v>460499.96</v>
+        <v>460499.93</v>
       </c>
       <c r="F130" s="8" t="n">
         <v>3897262.79</v>
@@ -9363,7 +9363,7 @@
         <v>-373564</v>
       </c>
       <c r="J130" s="9" t="n">
-        <v>834063.96</v>
+        <v>834063.9300000001</v>
       </c>
     </row>
     <row r="131">
@@ -9407,7 +9407,7 @@
         </is>
       </c>
       <c r="B132" s="9" t="n">
-        <v>466864.39</v>
+        <v>466864.4</v>
       </c>
       <c r="C132" s="9" t="n">
         <v>0</v>
@@ -9416,7 +9416,7 @@
         <v>0</v>
       </c>
       <c r="E132" s="9" t="n">
-        <v>466864.39</v>
+        <v>466864.4</v>
       </c>
       <c r="F132" s="8" t="n">
         <v>3897262.79</v>
@@ -9431,7 +9431,7 @@
         <v>-373564</v>
       </c>
       <c r="J132" s="9" t="n">
-        <v>840428.39</v>
+        <v>840428.4</v>
       </c>
     </row>
     <row r="133">
@@ -9441,7 +9441,7 @@
         </is>
       </c>
       <c r="B133" s="9" t="n">
-        <v>452670.71</v>
+        <v>452670.68</v>
       </c>
       <c r="C133" s="9" t="n">
         <v>0</v>
@@ -9450,7 +9450,7 @@
         <v>0</v>
       </c>
       <c r="E133" s="9" t="n">
-        <v>452670.71</v>
+        <v>452670.68</v>
       </c>
       <c r="F133" s="8" t="n">
         <v>3897262.79</v>
@@ -9465,7 +9465,7 @@
         <v>-373564</v>
       </c>
       <c r="J133" s="9" t="n">
-        <v>826234.71</v>
+        <v>826234.6800000001</v>
       </c>
     </row>
     <row r="134">
@@ -9475,7 +9475,7 @@
         </is>
       </c>
       <c r="B134" s="9" t="n">
-        <v>433657.62</v>
+        <v>433657.6</v>
       </c>
       <c r="C134" s="9" t="n">
         <v>0</v>
@@ -9484,7 +9484,7 @@
         <v>0</v>
       </c>
       <c r="E134" s="9" t="n">
-        <v>433657.62</v>
+        <v>433657.6</v>
       </c>
       <c r="F134" s="8" t="n">
         <v>3897262.79</v>
@@ -9499,7 +9499,7 @@
         <v>-373564</v>
       </c>
       <c r="J134" s="9" t="n">
-        <v>807221.62</v>
+        <v>807221.6</v>
       </c>
     </row>
     <row r="135">
@@ -9509,7 +9509,7 @@
         </is>
       </c>
       <c r="B135" s="9" t="n">
-        <v>440256.74</v>
+        <v>440256.72</v>
       </c>
       <c r="C135" s="9" t="n">
         <v>0</v>
@@ -9518,7 +9518,7 @@
         <v>0</v>
       </c>
       <c r="E135" s="9" t="n">
-        <v>440256.74</v>
+        <v>440256.72</v>
       </c>
       <c r="F135" s="8" t="n">
         <v>3897262.79</v>
@@ -9533,7 +9533,7 @@
         <v>-373564</v>
       </c>
       <c r="J135" s="9" t="n">
-        <v>813820.74</v>
+        <v>813820.72</v>
       </c>
     </row>
     <row r="136">
@@ -9543,7 +9543,7 @@
         </is>
       </c>
       <c r="B136" s="9" t="n">
-        <v>441870.6</v>
+        <v>441870.61</v>
       </c>
       <c r="C136" s="9" t="n">
         <v>0</v>
@@ -9552,7 +9552,7 @@
         <v>0</v>
       </c>
       <c r="E136" s="9" t="n">
-        <v>441870.6</v>
+        <v>441870.61</v>
       </c>
       <c r="F136" s="8" t="n">
         <v>3897262.79</v>
@@ -9567,7 +9567,7 @@
         <v>-373564</v>
       </c>
       <c r="J136" s="9" t="n">
-        <v>815434.6</v>
+        <v>815434.61</v>
       </c>
     </row>
     <row r="137">
@@ -9577,7 +9577,7 @@
         </is>
       </c>
       <c r="B137" s="9" t="n">
-        <v>444596.51</v>
+        <v>444596.47</v>
       </c>
       <c r="C137" s="9" t="n">
         <v>0</v>
@@ -9586,7 +9586,7 @@
         <v>0</v>
       </c>
       <c r="E137" s="9" t="n">
-        <v>444596.51</v>
+        <v>444596.47</v>
       </c>
       <c r="F137" s="8" t="n">
         <v>3897262.79</v>
@@ -9601,7 +9601,7 @@
         <v>-373564</v>
       </c>
       <c r="J137" s="9" t="n">
-        <v>818160.51</v>
+        <v>818160.47</v>
       </c>
     </row>
     <row r="138">
@@ -9645,7 +9645,7 @@
         </is>
       </c>
       <c r="B139" s="9" t="n">
-        <v>459043.57</v>
+        <v>459043.55</v>
       </c>
       <c r="C139" s="9" t="n">
         <v>0</v>
@@ -9654,7 +9654,7 @@
         <v>0</v>
       </c>
       <c r="E139" s="9" t="n">
-        <v>459043.57</v>
+        <v>459043.55</v>
       </c>
       <c r="F139" s="8" t="n">
         <v>3897262.79</v>
@@ -9669,7 +9669,7 @@
         <v>-373564</v>
       </c>
       <c r="J139" s="9" t="n">
-        <v>832607.5699999999</v>
+        <v>832607.55</v>
       </c>
     </row>
     <row r="140">
@@ -9815,7 +9815,7 @@
         </is>
       </c>
       <c r="B144" s="9" t="n">
-        <v>479303.95</v>
+        <v>479303.93</v>
       </c>
       <c r="C144" s="9" t="n">
         <v>0</v>
@@ -9824,7 +9824,7 @@
         <v>0</v>
       </c>
       <c r="E144" s="9" t="n">
-        <v>479303.95</v>
+        <v>479303.93</v>
       </c>
       <c r="F144" s="8" t="n">
         <v>3897262.79</v>
@@ -9839,7 +9839,7 @@
         <v>-373564</v>
       </c>
       <c r="J144" s="9" t="n">
-        <v>852867.95</v>
+        <v>852867.9300000001</v>
       </c>
     </row>
     <row r="145">
@@ -9849,7 +9849,7 @@
         </is>
       </c>
       <c r="B145" s="9" t="n">
-        <v>480848.73</v>
+        <v>480848.71</v>
       </c>
       <c r="C145" s="9" t="n">
         <v>0</v>
@@ -9858,7 +9858,7 @@
         <v>0</v>
       </c>
       <c r="E145" s="9" t="n">
-        <v>480848.73</v>
+        <v>480848.71</v>
       </c>
       <c r="F145" s="8" t="n">
         <v>3897262.79</v>
@@ -9873,7 +9873,7 @@
         <v>-373564</v>
       </c>
       <c r="J145" s="9" t="n">
-        <v>854412.73</v>
+        <v>854412.71</v>
       </c>
     </row>
     <row r="146">
@@ -9985,7 +9985,7 @@
         </is>
       </c>
       <c r="B149" s="9" t="n">
-        <v>502569.08</v>
+        <v>502070.76</v>
       </c>
       <c r="C149" s="9" t="n">
         <v>0</v>
@@ -9994,13 +9994,13 @@
         <v>0</v>
       </c>
       <c r="E149" s="9" t="n">
-        <v>502569.08</v>
+        <v>502070.76</v>
       </c>
       <c r="F149" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G149" s="16" t="n">
-        <v>0.128954</v>
+        <v>0.128827</v>
       </c>
       <c r="H149" s="9" t="n">
         <v>-0</v>
@@ -10009,7 +10009,7 @@
         <v>-382594</v>
       </c>
       <c r="J149" s="9" t="n">
-        <v>885163.08</v>
+        <v>884664.76</v>
       </c>
     </row>
     <row r="150">
@@ -10019,7 +10019,7 @@
         </is>
       </c>
       <c r="B150" s="9" t="n">
-        <v>509453.56</v>
+        <v>508656.68</v>
       </c>
       <c r="C150" s="9" t="n">
         <v>0</v>
@@ -10028,13 +10028,13 @@
         <v>0</v>
       </c>
       <c r="E150" s="9" t="n">
-        <v>509453.56</v>
+        <v>508656.68</v>
       </c>
       <c r="F150" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G150" s="16" t="n">
-        <v>0.130721</v>
+        <v>0.130516</v>
       </c>
       <c r="H150" s="9" t="n">
         <v>-0</v>
@@ -10043,7 +10043,7 @@
         <v>-382594</v>
       </c>
       <c r="J150" s="9" t="n">
-        <v>892047.5600000001</v>
+        <v>891250.6800000001</v>
       </c>
     </row>
     <row r="151">
@@ -10053,7 +10053,7 @@
         </is>
       </c>
       <c r="B151" s="9" t="n">
-        <v>516000.25</v>
+        <v>515501.92</v>
       </c>
       <c r="C151" s="9" t="n">
         <v>0</v>
@@ -10062,13 +10062,13 @@
         <v>0</v>
       </c>
       <c r="E151" s="9" t="n">
-        <v>516000.25</v>
+        <v>515501.92</v>
       </c>
       <c r="F151" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G151" s="16" t="n">
-        <v>0.132401</v>
+        <v>0.132273</v>
       </c>
       <c r="H151" s="9" t="n">
         <v>-0</v>
@@ -10077,7 +10077,7 @@
         <v>-340552</v>
       </c>
       <c r="J151" s="9" t="n">
-        <v>856552.25</v>
+        <v>856053.92</v>
       </c>
     </row>
     <row r="152">
@@ -10087,7 +10087,7 @@
         </is>
       </c>
       <c r="B152" s="9" t="n">
-        <v>518698.13</v>
+        <v>518597.9</v>
       </c>
       <c r="C152" s="9" t="n">
         <v>0</v>
@@ -10096,13 +10096,13 @@
         <v>0</v>
       </c>
       <c r="E152" s="9" t="n">
-        <v>518698.13</v>
+        <v>518597.9</v>
       </c>
       <c r="F152" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G152" s="16" t="n">
-        <v>0.133093</v>
+        <v>0.133067</v>
       </c>
       <c r="H152" s="9" t="n">
         <v>-0</v>
@@ -10111,7 +10111,7 @@
         <v>-340552</v>
       </c>
       <c r="J152" s="9" t="n">
-        <v>859250.13</v>
+        <v>859149.9</v>
       </c>
     </row>
     <row r="153">
@@ -10121,7 +10121,7 @@
         </is>
       </c>
       <c r="B153" s="9" t="n">
-        <v>526308.92</v>
+        <v>526905.37</v>
       </c>
       <c r="C153" s="9" t="n">
         <v>0</v>
@@ -10130,13 +10130,13 @@
         <v>0</v>
       </c>
       <c r="E153" s="9" t="n">
-        <v>526308.92</v>
+        <v>526905.37</v>
       </c>
       <c r="F153" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G153" s="16" t="n">
-        <v>0.135046</v>
+        <v>0.135199</v>
       </c>
       <c r="H153" s="9" t="n">
         <v>-0</v>
@@ -10145,7 +10145,7 @@
         <v>-380907</v>
       </c>
       <c r="J153" s="9" t="n">
-        <v>907215.92</v>
+        <v>907812.37</v>
       </c>
     </row>
     <row r="154">
@@ -10155,7 +10155,7 @@
         </is>
       </c>
       <c r="B154" s="9" t="n">
-        <v>528346.76</v>
+        <v>525360.3</v>
       </c>
       <c r="C154" s="9" t="n">
         <v>0</v>
@@ -10164,13 +10164,13 @@
         <v>0</v>
       </c>
       <c r="E154" s="9" t="n">
-        <v>528346.76</v>
+        <v>525360.3</v>
       </c>
       <c r="F154" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G154" s="16" t="n">
-        <v>0.135569</v>
+        <v>0.134802</v>
       </c>
       <c r="H154" s="9" t="n">
         <v>-0</v>
@@ -10179,7 +10179,7 @@
         <v>-380907</v>
       </c>
       <c r="J154" s="9" t="n">
-        <v>909253.76</v>
+        <v>906267.3</v>
       </c>
     </row>
     <row r="155">
@@ -10189,7 +10189,7 @@
         </is>
       </c>
       <c r="B155" s="9" t="n">
-        <v>531872.8</v>
+        <v>527094.91</v>
       </c>
       <c r="C155" s="9" t="n">
         <v>0</v>
@@ -10198,13 +10198,13 @@
         <v>0</v>
       </c>
       <c r="E155" s="9" t="n">
-        <v>531872.8</v>
+        <v>527094.91</v>
       </c>
       <c r="F155" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G155" s="16" t="n">
-        <v>0.136473</v>
+        <v>0.135247</v>
       </c>
       <c r="H155" s="9" t="n">
         <v>-0</v>
@@ -10213,7 +10213,7 @@
         <v>-380907</v>
       </c>
       <c r="J155" s="9" t="n">
-        <v>912779.8</v>
+        <v>908001.91</v>
       </c>
     </row>
     <row r="156">
@@ -10223,7 +10223,7 @@
         </is>
       </c>
       <c r="B156" s="9" t="n">
-        <v>547464.47</v>
+        <v>539800.33</v>
       </c>
       <c r="C156" s="9" t="n">
         <v>0</v>
@@ -10232,13 +10232,13 @@
         <v>0</v>
       </c>
       <c r="E156" s="9" t="n">
-        <v>547464.47</v>
+        <v>539800.33</v>
       </c>
       <c r="F156" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G156" s="16" t="n">
-        <v>0.140474</v>
+        <v>0.138508</v>
       </c>
       <c r="H156" s="9" t="n">
         <v>-0</v>
@@ -10247,7 +10247,7 @@
         <v>-302477</v>
       </c>
       <c r="J156" s="9" t="n">
-        <v>849941.47</v>
+        <v>842277.33</v>
       </c>
     </row>
     <row r="157">
@@ -10257,7 +10257,7 @@
         </is>
       </c>
       <c r="B157" s="9" t="n">
-        <v>550685.84</v>
+        <v>543021.71</v>
       </c>
       <c r="C157" s="9" t="n">
         <v>0</v>
@@ -10266,13 +10266,13 @@
         <v>0</v>
       </c>
       <c r="E157" s="9" t="n">
-        <v>550685.84</v>
+        <v>543021.71</v>
       </c>
       <c r="F157" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G157" s="16" t="n">
-        <v>0.141301</v>
+        <v>0.139334</v>
       </c>
       <c r="H157" s="9" t="n">
         <v>-0</v>
@@ -10281,7 +10281,7 @@
         <v>-269477</v>
       </c>
       <c r="J157" s="9" t="n">
-        <v>820162.84</v>
+        <v>812498.71</v>
       </c>
     </row>
     <row r="158">
@@ -10291,7 +10291,7 @@
         </is>
       </c>
       <c r="B158" s="9" t="n">
-        <v>547246.2</v>
+        <v>538885.4</v>
       </c>
       <c r="C158" s="9" t="n">
         <v>0</v>
@@ -10300,13 +10300,13 @@
         <v>0</v>
       </c>
       <c r="E158" s="9" t="n">
-        <v>547246.2</v>
+        <v>538885.4</v>
       </c>
       <c r="F158" s="8" t="n">
         <v>3897262.79</v>
       </c>
       <c r="G158" s="16" t="n">
-        <v>0.140418</v>
+        <v>0.138273</v>
       </c>
       <c r="H158" s="9" t="n">
         <v>-0</v>
@@ -10315,7 +10315,7 @@
         <v>-269477</v>
       </c>
       <c r="J158" s="9" t="n">
-        <v>816723.2</v>
+        <v>808362.4</v>
       </c>
     </row>
     <row r="159">
@@ -10563,7 +10563,7 @@
         </is>
       </c>
       <c r="B166" s="9" t="n">
-        <v>106685.82</v>
+        <v>106685.81</v>
       </c>
       <c r="C166" s="9" t="n">
         <v>0</v>
@@ -10572,7 +10572,7 @@
         <v>0</v>
       </c>
       <c r="E166" s="9" t="n">
-        <v>106685.82</v>
+        <v>106685.81</v>
       </c>
       <c r="F166" s="8" t="n">
         <v>745251.28</v>
@@ -10587,7 +10587,7 @@
         <v>-43462</v>
       </c>
       <c r="J166" s="9" t="n">
-        <v>150147.82</v>
+        <v>150147.81</v>
       </c>
     </row>
     <row r="167">
@@ -10699,7 +10699,7 @@
         </is>
       </c>
       <c r="B170" s="9" t="n">
-        <v>104908.98</v>
+        <v>104908.99</v>
       </c>
       <c r="C170" s="9" t="n">
         <v>0</v>
@@ -10708,7 +10708,7 @@
         <v>0</v>
       </c>
       <c r="E170" s="9" t="n">
-        <v>104908.98</v>
+        <v>104908.99</v>
       </c>
       <c r="F170" s="8" t="n">
         <v>745251.28</v>
@@ -10723,7 +10723,7 @@
         <v>-43462</v>
       </c>
       <c r="J170" s="9" t="n">
-        <v>148370.98</v>
+        <v>148370.99</v>
       </c>
     </row>
     <row r="171">
@@ -10733,7 +10733,7 @@
         </is>
       </c>
       <c r="B171" s="9" t="n">
-        <v>101994.86</v>
+        <v>101994.85</v>
       </c>
       <c r="C171" s="9" t="n">
         <v>0</v>
@@ -10742,7 +10742,7 @@
         <v>0</v>
       </c>
       <c r="E171" s="9" t="n">
-        <v>101994.86</v>
+        <v>101994.85</v>
       </c>
       <c r="F171" s="8" t="n">
         <v>745251.28</v>
@@ -10757,7 +10757,7 @@
         <v>-43462</v>
       </c>
       <c r="J171" s="9" t="n">
-        <v>145456.86</v>
+        <v>145456.85</v>
       </c>
     </row>
     <row r="172">
@@ -10835,7 +10835,7 @@
         </is>
       </c>
       <c r="B174" s="9" t="n">
-        <v>101961.08</v>
+        <v>101961.07</v>
       </c>
       <c r="C174" s="9" t="n">
         <v>0</v>
@@ -10844,7 +10844,7 @@
         <v>0</v>
       </c>
       <c r="E174" s="9" t="n">
-        <v>101961.08</v>
+        <v>101961.07</v>
       </c>
       <c r="F174" s="8" t="n">
         <v>745251.28</v>
@@ -10859,7 +10859,7 @@
         <v>-59392</v>
       </c>
       <c r="J174" s="9" t="n">
-        <v>161353.08</v>
+        <v>161353.07</v>
       </c>
     </row>
     <row r="175">
@@ -10971,7 +10971,7 @@
         </is>
       </c>
       <c r="B178" s="9" t="n">
-        <v>250873.73</v>
+        <v>250873.74</v>
       </c>
       <c r="C178" s="9" t="n">
         <v>0</v>
@@ -10980,7 +10980,7 @@
         <v>0</v>
       </c>
       <c r="E178" s="9" t="n">
-        <v>250873.73</v>
+        <v>250873.74</v>
       </c>
       <c r="F178" s="8" t="n">
         <v>1905830.74</v>
@@ -10995,7 +10995,7 @@
         <v>-12014</v>
       </c>
       <c r="J178" s="9" t="n">
-        <v>262887.73</v>
+        <v>262887.74</v>
       </c>
     </row>
     <row r="179">
@@ -11107,7 +11107,7 @@
         </is>
       </c>
       <c r="B182" s="9" t="n">
-        <v>257851.67</v>
+        <v>257851.68</v>
       </c>
       <c r="C182" s="9" t="n">
         <v>0</v>
@@ -11116,7 +11116,7 @@
         <v>0</v>
       </c>
       <c r="E182" s="9" t="n">
-        <v>257851.67</v>
+        <v>257851.68</v>
       </c>
       <c r="F182" s="8" t="n">
         <v>1905830.74</v>
@@ -11131,7 +11131,7 @@
         <v>-12014</v>
       </c>
       <c r="J182" s="9" t="n">
-        <v>269865.67</v>
+        <v>269865.68</v>
       </c>
     </row>
     <row r="183">
@@ -11277,7 +11277,7 @@
         </is>
       </c>
       <c r="B187" s="9" t="n">
-        <v>268045.03</v>
+        <v>268045.02</v>
       </c>
       <c r="C187" s="9" t="n">
         <v>0</v>
@@ -11286,7 +11286,7 @@
         <v>0</v>
       </c>
       <c r="E187" s="9" t="n">
-        <v>268045.03</v>
+        <v>268045.02</v>
       </c>
       <c r="F187" s="8" t="n">
         <v>1905830.74</v>
@@ -11301,7 +11301,7 @@
         <v>-12014</v>
       </c>
       <c r="J187" s="9" t="n">
-        <v>280059.03</v>
+        <v>280059.02</v>
       </c>
     </row>
     <row r="188">
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="B189" s="9" t="n">
-        <v>272955.59</v>
+        <v>272955.6</v>
       </c>
       <c r="C189" s="9" t="n">
         <v>0</v>
@@ -11354,7 +11354,7 @@
         <v>0</v>
       </c>
       <c r="E189" s="9" t="n">
-        <v>272955.59</v>
+        <v>272955.6</v>
       </c>
       <c r="F189" s="8" t="n">
         <v>1905830.74</v>
@@ -11369,7 +11369,7 @@
         <v>-12014</v>
       </c>
       <c r="J189" s="9" t="n">
-        <v>284969.59</v>
+        <v>284969.6</v>
       </c>
     </row>
     <row r="190">
@@ -11515,7 +11515,7 @@
         </is>
       </c>
       <c r="B194" s="9" t="n">
-        <v>283408.73</v>
+        <v>283408.72</v>
       </c>
       <c r="C194" s="9" t="n">
         <v>0</v>
@@ -11524,7 +11524,7 @@
         <v>0</v>
       </c>
       <c r="E194" s="9" t="n">
-        <v>283408.73</v>
+        <v>283408.72</v>
       </c>
       <c r="F194" s="8" t="n">
         <v>1905830.74</v>
@@ -11539,7 +11539,7 @@
         <v>-12014</v>
       </c>
       <c r="J194" s="9" t="n">
-        <v>295422.73</v>
+        <v>295422.72</v>
       </c>
     </row>
     <row r="195">
@@ -11617,7 +11617,7 @@
         </is>
       </c>
       <c r="B197" s="9" t="n">
-        <v>269528.2</v>
+        <v>269528.19</v>
       </c>
       <c r="C197" s="9" t="n">
         <v>0</v>
@@ -11626,7 +11626,7 @@
         <v>0</v>
       </c>
       <c r="E197" s="9" t="n">
-        <v>269528.2</v>
+        <v>269528.19</v>
       </c>
       <c r="F197" s="8" t="n">
         <v>1905830.74</v>
@@ -11641,7 +11641,7 @@
         <v>-12014</v>
       </c>
       <c r="J197" s="9" t="n">
-        <v>281542.2</v>
+        <v>281542.19</v>
       </c>
     </row>
     <row r="198">
@@ -11719,7 +11719,7 @@
         </is>
       </c>
       <c r="B200" s="9" t="n">
-        <v>261000.91</v>
+        <v>261000.9</v>
       </c>
       <c r="C200" s="9" t="n">
         <v>0</v>
@@ -11728,7 +11728,7 @@
         <v>0</v>
       </c>
       <c r="E200" s="9" t="n">
-        <v>261000.91</v>
+        <v>261000.9</v>
       </c>
       <c r="F200" s="8" t="n">
         <v>1905830.74</v>
@@ -11743,7 +11743,7 @@
         <v>-34394</v>
       </c>
       <c r="J200" s="9" t="n">
-        <v>295394.91</v>
+        <v>295394.9</v>
       </c>
     </row>
     <row r="201">
@@ -11787,7 +11787,7 @@
         </is>
       </c>
       <c r="B202" s="9" t="n">
-        <v>267401.95</v>
+        <v>267401.94</v>
       </c>
       <c r="C202" s="9" t="n">
         <v>0</v>
@@ -11796,7 +11796,7 @@
         <v>0</v>
       </c>
       <c r="E202" s="9" t="n">
-        <v>267401.95</v>
+        <v>267401.94</v>
       </c>
       <c r="F202" s="8" t="n">
         <v>1905830.74</v>
@@ -11811,7 +11811,7 @@
         <v>-34394</v>
       </c>
       <c r="J202" s="9" t="n">
-        <v>301795.95</v>
+        <v>301795.94</v>
       </c>
     </row>
     <row r="203">
@@ -12365,7 +12365,7 @@
         </is>
       </c>
       <c r="B219" s="9" t="n">
-        <v>292136.17</v>
+        <v>292136.18</v>
       </c>
       <c r="C219" s="9" t="n">
         <v>0</v>
@@ -12374,7 +12374,7 @@
         <v>0</v>
       </c>
       <c r="E219" s="9" t="n">
-        <v>292136.17</v>
+        <v>292136.18</v>
       </c>
       <c r="F219" s="8" t="n">
         <v>1905830.74</v>
@@ -12389,7 +12389,7 @@
         <v>78146</v>
       </c>
       <c r="J219" s="9" t="n">
-        <v>213990.17</v>
+        <v>213990.18</v>
       </c>
     </row>
     <row r="220">
@@ -17057,7 +17057,7 @@
         </is>
       </c>
       <c r="B357" s="9" t="n">
-        <v>284366.01</v>
+        <v>285941</v>
       </c>
       <c r="C357" s="9" t="n">
         <v>0</v>
@@ -17066,13 +17066,13 @@
         <v>0</v>
       </c>
       <c r="E357" s="9" t="n">
-        <v>284366.01</v>
+        <v>285941</v>
       </c>
       <c r="F357" s="8" t="n">
         <v>1905830.74</v>
       </c>
       <c r="G357" s="16" t="n">
-        <v>0.149208</v>
+        <v>0.150035</v>
       </c>
       <c r="H357" s="9" t="n">
         <v>-0</v>
@@ -17081,7 +17081,41 @@
         <v>-138224</v>
       </c>
       <c r="J357" s="9" t="n">
-        <v>422590.01</v>
+        <v>424165</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="B358" s="9" t="n">
+        <v>297886</v>
+      </c>
+      <c r="C358" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D358" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E358" s="9" t="n">
+        <v>297886</v>
+      </c>
+      <c r="F358" s="8" t="n">
+        <v>1905830.74</v>
+      </c>
+      <c r="G358" s="16" t="n">
+        <v>0.156302</v>
+      </c>
+      <c r="H358" s="9" t="n">
+        <v>-0</v>
+      </c>
+      <c r="I358" s="9" t="n">
+        <v>-138224</v>
+      </c>
+      <c r="J358" s="9" t="n">
+        <v>436110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>